<commit_message>
update excel upload score
</commit_message>
<xml_diff>
--- a/src/assets/templates/Template-uploadStudentScore.xlsx
+++ b/src/assets/templates/Template-uploadStudentScore.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D448B77-4492-4D03-8577-8F83801E803C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B325C6FA-88FF-4354-8583-665CCCE0131A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A892E446-8B98-49BD-9081-538FFC902A6D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{A892E446-8B98-49BD-9081-538FFC902A6D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="ข้อมูล Dropdown" sheetId="2" r:id="rId2"/>
+    <sheet name="split-ชื่อนิสิต" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="38">
   <si>
     <t>ลำดับ</t>
   </si>
@@ -253,12 +254,57 @@
       <t>-</t>
     </r>
   </si>
+  <si>
+    <t>นายสมชาย ใจดี</t>
+  </si>
+  <si>
+    <t>เครื่องมือแยกคำนำหน้าและชื่อนิสิต</t>
+  </si>
+  <si>
+    <t>ข้อความที่ต้องการแยก</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">วิธีใช้งาน </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>กรอกชื่อที่ต้องการแยก</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="3"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ใน Column A</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">แล้วจะได้ - คำนำหน้า ใน Column B </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                       - ชื่อ-นามสกุล ใน Column C</t>
+  </si>
+  <si>
+    <t>สามารถคัดลอกไปใส่ในรายชื่อใน Sheet1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -310,8 +356,48 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -324,8 +410,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -333,19 +437,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -781,7 +914,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C2" t="s">
@@ -793,7 +926,7 @@
       <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" t="s">
         <v>27</v>
       </c>
       <c r="G2">
@@ -805,20 +938,20 @@
       <c r="I2">
         <v>45</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C3" t="s">
@@ -830,7 +963,7 @@
       <c r="E3" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" t="s">
         <v>28</v>
       </c>
       <c r="H3">
@@ -839,14 +972,14 @@
       <c r="I3">
         <v>30</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -955,6 +1088,1175 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9793ADFD-2ECD-45F7-A650-5D55AD0BA584}">
+  <dimension ref="A1:H102"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="21.88671875" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="9" t="str">
+        <f>IF(OR(LEFT(A3,3)="นาย",LEFT(A3,3)="นาง"),LEFT(A3,3),IF(LEFT(A3,6)="นางสาว",LEFT(A3,6),""))</f>
+        <v>นาย</v>
+      </c>
+      <c r="C3" s="9" t="str">
+        <f>TRIM(SUBSTITUTE(A3,B3,""))</f>
+        <v>สมชาย ใจดี</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9" t="str">
+        <f t="shared" ref="B4:B67" si="0">IF(OR(LEFT(A4,3)="นาย",LEFT(A4,3)="นาง"),LEFT(A4,3),IF(LEFT(A4,6)="นางสาว",LEFT(A4,6),""))</f>
+        <v/>
+      </c>
+      <c r="C4" s="9" t="str">
+        <f t="shared" ref="C4:C20" si="1">TRIM(SUBSTITUTE(A4,B4,""))</f>
+        <v/>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C5" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C6" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C7" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C8" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="B9" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C9" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C10" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C11" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="9"/>
+      <c r="B12" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C12" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C13" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="9"/>
+      <c r="B14" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C14" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C15" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C16" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C17" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="9"/>
+      <c r="B18" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C18" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="9"/>
+      <c r="B19" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C19" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="9"/>
+      <c r="B20" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C20" s="9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="9"/>
+      <c r="B21" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C21" s="9" t="str">
+        <f t="shared" ref="C21:C41" si="2">TRIM(SUBSTITUTE(A21,B21,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="9"/>
+      <c r="B22" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C22" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="9"/>
+      <c r="B23" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C23" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="9"/>
+      <c r="B24" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C24" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="9"/>
+      <c r="B25" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C25" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="9"/>
+      <c r="B26" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C26" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="9"/>
+      <c r="B27" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C27" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="9"/>
+      <c r="B28" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C28" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="9"/>
+      <c r="B29" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C29" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="9"/>
+      <c r="B30" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C30" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="9"/>
+      <c r="B31" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C31" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="9"/>
+      <c r="B32" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C32" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="9"/>
+      <c r="B33" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C33" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="9"/>
+      <c r="B34" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C34" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="9"/>
+      <c r="B35" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C35" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="9"/>
+      <c r="B36" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C36" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="9"/>
+      <c r="B37" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C37" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="9"/>
+      <c r="B38" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C38" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="9"/>
+      <c r="B39" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C39" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="9"/>
+      <c r="B40" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C40" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="9"/>
+      <c r="B41" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C41" s="9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="9"/>
+      <c r="B42" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C42" s="9" t="str">
+        <f t="shared" ref="C42:C102" si="3">TRIM(SUBSTITUTE(A42,B42,""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="9"/>
+      <c r="B43" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C43" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="9"/>
+      <c r="B44" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C44" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="9"/>
+      <c r="B45" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C45" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="9"/>
+      <c r="B46" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C46" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="9"/>
+      <c r="B47" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C47" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="9"/>
+      <c r="B48" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C48" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="9"/>
+      <c r="B49" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C49" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="9"/>
+      <c r="B50" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C50" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="9"/>
+      <c r="B51" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C51" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="9"/>
+      <c r="B52" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C52" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="9"/>
+      <c r="B53" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C53" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="9"/>
+      <c r="B54" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C54" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="9"/>
+      <c r="B55" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C55" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" s="9"/>
+      <c r="B56" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C56" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" s="9"/>
+      <c r="B57" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C57" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="9"/>
+      <c r="B58" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C58" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="9"/>
+      <c r="B59" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C59" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="9"/>
+      <c r="B60" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C60" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="9"/>
+      <c r="B61" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C61" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="9"/>
+      <c r="B62" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C62" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" s="9"/>
+      <c r="B63" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C63" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" s="9"/>
+      <c r="B64" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C64" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="9"/>
+      <c r="B65" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C65" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="9"/>
+      <c r="B66" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C66" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="9"/>
+      <c r="B67" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C67" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="9"/>
+      <c r="B68" s="9" t="str">
+        <f t="shared" ref="B68:B102" si="4">IF(OR(LEFT(A68,3)="นาย",LEFT(A68,3)="นาง"),LEFT(A68,3),IF(LEFT(A68,6)="นางสาว",LEFT(A68,6),""))</f>
+        <v/>
+      </c>
+      <c r="C68" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="9"/>
+      <c r="B69" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C69" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="9"/>
+      <c r="B70" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C70" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="9"/>
+      <c r="B71" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C71" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="9"/>
+      <c r="B72" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C72" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="9"/>
+      <c r="B73" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C73" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="9"/>
+      <c r="B74" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C74" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="9"/>
+      <c r="B75" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C75" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="9"/>
+      <c r="B76" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C76" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="9"/>
+      <c r="B77" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C77" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="9"/>
+      <c r="B78" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C78" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="9"/>
+      <c r="B79" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C79" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="9"/>
+      <c r="B80" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C80" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="9"/>
+      <c r="B81" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C81" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" s="9"/>
+      <c r="B82" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C82" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" s="9"/>
+      <c r="B83" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C83" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A84" s="9"/>
+      <c r="B84" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C84" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="9"/>
+      <c r="B85" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C85" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" s="9"/>
+      <c r="B86" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C86" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" s="9"/>
+      <c r="B87" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C87" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="9"/>
+      <c r="B88" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C88" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A89" s="9"/>
+      <c r="B89" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C89" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="9"/>
+      <c r="B90" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C90" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="9"/>
+      <c r="B91" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C91" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" s="9"/>
+      <c r="B92" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C92" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" s="9"/>
+      <c r="B93" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C93" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="9"/>
+      <c r="B94" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C94" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="9"/>
+      <c r="B95" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C95" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96" s="9"/>
+      <c r="B96" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C96" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" s="9"/>
+      <c r="B97" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C97" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A98" s="9"/>
+      <c r="B98" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C98" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99" s="9"/>
+      <c r="B99" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C99" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" s="9"/>
+      <c r="B100" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C100" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A101" s="9"/>
+      <c r="B101" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C101" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A102" s="9"/>
+      <c r="B102" s="9" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C102" s="9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="E3:H3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1201,20 +2503,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1237,26 +2539,26 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCB6AB14-C0AE-473C-89A3-515A96D03C50}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="6e8d88bf-11ac-458b-86c1-bcd44f8a4dcf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66F9059C-B81D-4D59-AB43-86C418F000DC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCB6AB14-C0AE-473C-89A3-515A96D03C50}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="6e8d88bf-11ac-458b-86c1-bcd44f8a4dcf"/>
-    <ds:schemaRef ds:uri="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
change current page to sheet1
</commit_message>
<xml_diff>
--- a/src/assets/templates/Template-uploadStudentScore.xlsx
+++ b/src/assets/templates/Template-uploadStudentScore.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SourceTree\score-management\src\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B325C6FA-88FF-4354-8583-665CCCE0131A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45363291-FB48-43DD-9F38-651923530AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{A892E446-8B98-49BD-9081-538FFC902A6D}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8880" xr2:uid="{A892E446-8B98-49BD-9081-538FFC902A6D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -456,19 +456,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -477,8 +472,12 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -518,10 +517,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -938,14 +933,14 @@
       <c r="I2">
         <v>45</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3">
@@ -972,14 +967,14 @@
       <c r="I3">
         <v>30</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1105,1146 +1100,1145 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="7" t="s">
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="E1" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="9" t="str">
+      <c r="B3" s="3" t="str">
         <f>IF(OR(LEFT(A3,3)="นาย",LEFT(A3,3)="นาง"),LEFT(A3,3),IF(LEFT(A3,6)="นางสาว",LEFT(A3,6),""))</f>
         <v>นาย</v>
       </c>
-      <c r="C3" s="9" t="str">
+      <c r="C3" s="3" t="str">
         <f>TRIM(SUBSTITUTE(A3,B3,""))</f>
         <v>สมชาย ใจดี</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9" t="str">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3" t="str">
         <f t="shared" ref="B4:B67" si="0">IF(OR(LEFT(A4,3)="นาย",LEFT(A4,3)="นาง"),LEFT(A4,3),IF(LEFT(A4,6)="นางสาว",LEFT(A4,6),""))</f>
         <v/>
       </c>
-      <c r="C4" s="9" t="str">
+      <c r="C4" s="3" t="str">
         <f t="shared" ref="C4:C20" si="1">TRIM(SUBSTITUTE(A4,B4,""))</f>
         <v/>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C5" s="9" t="str">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C5" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C6" s="9" t="str">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C6" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C7" s="9" t="str">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C7" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C8" s="9" t="str">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C8" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C9" s="9" t="str">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C9" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C10" s="9" t="str">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C10" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C11" s="9" t="str">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C11" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C12" s="9" t="str">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C12" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C13" s="9" t="str">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C13" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C14" s="9" t="str">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C14" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C15" s="9" t="str">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C15" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C16" s="9" t="str">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C16" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C17" s="9" t="str">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C17" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C18" s="9" t="str">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C18" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C19" s="9" t="str">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C19" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C20" s="9" t="str">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C20" s="3" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C21" s="9" t="str">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C21" s="3" t="str">
         <f t="shared" ref="C21:C41" si="2">TRIM(SUBSTITUTE(A21,B21,""))</f>
         <v/>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C22" s="9" t="str">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C22" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C23" s="9" t="str">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C23" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C24" s="9" t="str">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C24" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C25" s="9" t="str">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C25" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C26" s="9" t="str">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C26" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="9"/>
-      <c r="B27" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C27" s="9" t="str">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C27" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C28" s="9" t="str">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C28" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="9"/>
-      <c r="B29" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C29" s="9" t="str">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C29" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C30" s="9" t="str">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C30" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="9"/>
-      <c r="B31" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C31" s="9" t="str">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C31" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="9"/>
-      <c r="B32" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C32" s="9" t="str">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C32" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="9"/>
-      <c r="B33" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C33" s="9" t="str">
+      <c r="A33" s="3"/>
+      <c r="B33" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C33" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="9"/>
-      <c r="B34" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C34" s="9" t="str">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C34" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="9"/>
-      <c r="B35" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C35" s="9" t="str">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C35" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="9"/>
-      <c r="B36" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C36" s="9" t="str">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C36" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="9"/>
-      <c r="B37" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C37" s="9" t="str">
+      <c r="A37" s="3"/>
+      <c r="B37" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C37" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="9"/>
-      <c r="B38" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C38" s="9" t="str">
+      <c r="A38" s="3"/>
+      <c r="B38" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C38" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="9"/>
-      <c r="B39" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C39" s="9" t="str">
+      <c r="A39" s="3"/>
+      <c r="B39" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C39" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="9"/>
-      <c r="B40" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C40" s="9" t="str">
+      <c r="A40" s="3"/>
+      <c r="B40" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C40" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="9"/>
-      <c r="B41" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C41" s="9" t="str">
+      <c r="A41" s="3"/>
+      <c r="B41" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C41" s="3" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="9"/>
-      <c r="B42" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C42" s="9" t="str">
+      <c r="A42" s="3"/>
+      <c r="B42" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C42" s="3" t="str">
         <f t="shared" ref="C42:C102" si="3">TRIM(SUBSTITUTE(A42,B42,""))</f>
         <v/>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="9"/>
-      <c r="B43" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C43" s="9" t="str">
+      <c r="A43" s="3"/>
+      <c r="B43" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C43" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="9"/>
-      <c r="B44" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C44" s="9" t="str">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C44" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="9"/>
-      <c r="B45" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C45" s="9" t="str">
+      <c r="A45" s="3"/>
+      <c r="B45" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C45" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="9"/>
-      <c r="B46" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C46" s="9" t="str">
+      <c r="A46" s="3"/>
+      <c r="B46" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C46" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="9"/>
-      <c r="B47" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C47" s="9" t="str">
+      <c r="A47" s="3"/>
+      <c r="B47" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C47" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="9"/>
-      <c r="B48" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C48" s="9" t="str">
+      <c r="A48" s="3"/>
+      <c r="B48" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C48" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="9"/>
-      <c r="B49" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C49" s="9" t="str">
+      <c r="A49" s="3"/>
+      <c r="B49" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C49" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="9"/>
-      <c r="B50" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C50" s="9" t="str">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C50" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="9"/>
-      <c r="B51" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C51" s="9" t="str">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C51" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="9"/>
-      <c r="B52" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C52" s="9" t="str">
+      <c r="A52" s="3"/>
+      <c r="B52" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C52" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="9"/>
-      <c r="B53" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C53" s="9" t="str">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C53" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="9"/>
-      <c r="B54" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C54" s="9" t="str">
+      <c r="A54" s="3"/>
+      <c r="B54" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C54" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="9"/>
-      <c r="B55" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C55" s="9" t="str">
+      <c r="A55" s="3"/>
+      <c r="B55" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C55" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="9"/>
-      <c r="B56" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C56" s="9" t="str">
+      <c r="A56" s="3"/>
+      <c r="B56" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C56" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="9"/>
-      <c r="B57" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C57" s="9" t="str">
+      <c r="A57" s="3"/>
+      <c r="B57" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C57" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="9"/>
-      <c r="B58" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C58" s="9" t="str">
+      <c r="A58" s="3"/>
+      <c r="B58" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C58" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="9"/>
-      <c r="B59" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C59" s="9" t="str">
+      <c r="A59" s="3"/>
+      <c r="B59" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C59" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="9"/>
-      <c r="B60" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C60" s="9" t="str">
+      <c r="A60" s="3"/>
+      <c r="B60" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C60" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="9"/>
-      <c r="B61" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C61" s="9" t="str">
+      <c r="A61" s="3"/>
+      <c r="B61" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C61" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="9"/>
-      <c r="B62" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C62" s="9" t="str">
+      <c r="A62" s="3"/>
+      <c r="B62" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C62" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="9"/>
-      <c r="B63" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C63" s="9" t="str">
+      <c r="A63" s="3"/>
+      <c r="B63" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C63" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="9"/>
-      <c r="B64" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C64" s="9" t="str">
+      <c r="A64" s="3"/>
+      <c r="B64" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C64" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="9"/>
-      <c r="B65" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C65" s="9" t="str">
+      <c r="A65" s="3"/>
+      <c r="B65" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C65" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="9"/>
-      <c r="B66" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C66" s="9" t="str">
+      <c r="A66" s="3"/>
+      <c r="B66" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C66" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="9"/>
-      <c r="B67" s="9" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="C67" s="9" t="str">
+      <c r="A67" s="3"/>
+      <c r="B67" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C67" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="9"/>
-      <c r="B68" s="9" t="str">
+      <c r="A68" s="3"/>
+      <c r="B68" s="3" t="str">
         <f t="shared" ref="B68:B102" si="4">IF(OR(LEFT(A68,3)="นาย",LEFT(A68,3)="นาง"),LEFT(A68,3),IF(LEFT(A68,6)="นางสาว",LEFT(A68,6),""))</f>
         <v/>
       </c>
-      <c r="C68" s="9" t="str">
+      <c r="C68" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="9"/>
-      <c r="B69" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C69" s="9" t="str">
+      <c r="A69" s="3"/>
+      <c r="B69" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C69" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="9"/>
-      <c r="B70" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C70" s="9" t="str">
+      <c r="A70" s="3"/>
+      <c r="B70" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C70" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="9"/>
-      <c r="B71" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C71" s="9" t="str">
+      <c r="A71" s="3"/>
+      <c r="B71" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C71" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="9"/>
-      <c r="B72" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C72" s="9" t="str">
+      <c r="A72" s="3"/>
+      <c r="B72" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C72" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="9"/>
-      <c r="B73" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C73" s="9" t="str">
+      <c r="A73" s="3"/>
+      <c r="B73" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C73" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A74" s="9"/>
-      <c r="B74" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C74" s="9" t="str">
+      <c r="A74" s="3"/>
+      <c r="B74" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C74" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A75" s="9"/>
-      <c r="B75" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C75" s="9" t="str">
+      <c r="A75" s="3"/>
+      <c r="B75" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C75" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A76" s="9"/>
-      <c r="B76" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C76" s="9" t="str">
+      <c r="A76" s="3"/>
+      <c r="B76" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C76" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A77" s="9"/>
-      <c r="B77" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C77" s="9" t="str">
+      <c r="A77" s="3"/>
+      <c r="B77" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C77" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A78" s="9"/>
-      <c r="B78" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C78" s="9" t="str">
+      <c r="A78" s="3"/>
+      <c r="B78" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C78" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A79" s="9"/>
-      <c r="B79" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C79" s="9" t="str">
+      <c r="A79" s="3"/>
+      <c r="B79" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C79" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A80" s="9"/>
-      <c r="B80" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C80" s="9" t="str">
+      <c r="A80" s="3"/>
+      <c r="B80" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C80" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A81" s="9"/>
-      <c r="B81" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C81" s="9" t="str">
+      <c r="A81" s="3"/>
+      <c r="B81" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C81" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A82" s="9"/>
-      <c r="B82" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C82" s="9" t="str">
+      <c r="A82" s="3"/>
+      <c r="B82" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C82" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A83" s="9"/>
-      <c r="B83" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C83" s="9" t="str">
+      <c r="A83" s="3"/>
+      <c r="B83" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C83" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A84" s="9"/>
-      <c r="B84" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C84" s="9" t="str">
+      <c r="A84" s="3"/>
+      <c r="B84" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C84" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A85" s="9"/>
-      <c r="B85" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C85" s="9" t="str">
+      <c r="A85" s="3"/>
+      <c r="B85" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C85" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A86" s="9"/>
-      <c r="B86" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C86" s="9" t="str">
+      <c r="A86" s="3"/>
+      <c r="B86" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C86" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A87" s="9"/>
-      <c r="B87" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C87" s="9" t="str">
+      <c r="A87" s="3"/>
+      <c r="B87" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C87" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A88" s="9"/>
-      <c r="B88" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C88" s="9" t="str">
+      <c r="A88" s="3"/>
+      <c r="B88" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C88" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A89" s="9"/>
-      <c r="B89" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C89" s="9" t="str">
+      <c r="A89" s="3"/>
+      <c r="B89" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C89" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A90" s="9"/>
-      <c r="B90" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C90" s="9" t="str">
+      <c r="A90" s="3"/>
+      <c r="B90" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C90" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A91" s="9"/>
-      <c r="B91" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C91" s="9" t="str">
+      <c r="A91" s="3"/>
+      <c r="B91" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C91" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A92" s="9"/>
-      <c r="B92" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C92" s="9" t="str">
+      <c r="A92" s="3"/>
+      <c r="B92" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C92" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A93" s="9"/>
-      <c r="B93" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C93" s="9" t="str">
+      <c r="A93" s="3"/>
+      <c r="B93" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C93" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A94" s="9"/>
-      <c r="B94" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C94" s="9" t="str">
+      <c r="A94" s="3"/>
+      <c r="B94" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C94" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A95" s="9"/>
-      <c r="B95" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C95" s="9" t="str">
+      <c r="A95" s="3"/>
+      <c r="B95" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C95" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A96" s="9"/>
-      <c r="B96" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C96" s="9" t="str">
+      <c r="A96" s="3"/>
+      <c r="B96" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C96" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A97" s="9"/>
-      <c r="B97" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C97" s="9" t="str">
+      <c r="A97" s="3"/>
+      <c r="B97" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C97" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A98" s="9"/>
-      <c r="B98" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C98" s="9" t="str">
+      <c r="A98" s="3"/>
+      <c r="B98" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C98" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A99" s="9"/>
-      <c r="B99" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C99" s="9" t="str">
+      <c r="A99" s="3"/>
+      <c r="B99" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C99" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A100" s="9"/>
-      <c r="B100" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C100" s="9" t="str">
+      <c r="A100" s="3"/>
+      <c r="B100" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C100" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A101" s="9"/>
-      <c r="B101" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C101" s="9" t="str">
+      <c r="A101" s="3"/>
+      <c r="B101" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C101" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A102" s="9"/>
-      <c r="B102" s="9" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="C102" s="9" t="str">
+      <c r="A102" s="3"/>
+      <c r="B102" s="3" t="str">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="C102" s="3" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
@@ -2262,6 +2256,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100479A8332356E304793497BBC6982E2EA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="38024756525751a81199743b20bc73d7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d" xmlns:ns4="6e8d88bf-11ac-458b-86c1-bcd44f8a4dcf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3aa9a955e580ac50f8fdc526b3761519" ns3:_="" ns4:_="">
     <xsd:import namespace="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d"/>
@@ -2502,14 +2504,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2520,6 +2514,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCB6AB14-C0AE-473C-89A3-515A96D03C50}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="6e8d88bf-11ac-458b-86c1-bcd44f8a4dcf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F50997C-82B0-4661-81F0-206B60F6EA3C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2538,23 +2549,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCB6AB14-C0AE-473C-89A3-515A96D03C50}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="5f57a6f6-9a89-4746-97fb-1b0e2ec9618d"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="6e8d88bf-11ac-458b-86c1-bcd44f8a4dcf"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66F9059C-B81D-4D59-AB43-86C418F000DC}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
excel uploadScore protect edit column name
</commit_message>
<xml_diff>
--- a/src/assets/templates/Template-uploadStudentScore.xlsx
+++ b/src/assets/templates/Template-uploadStudentScore.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ReportScore\Present\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F2741C-2F42-4243-AFA8-DE634E4D0FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4CC61AF-67BF-4C79-8534-E92D09309ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A892E446-8B98-49BD-9081-538FFC902A6D}"/>
   </bookViews>
@@ -369,29 +369,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
+      <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="10">
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -405,12 +427,27 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -426,7 +463,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AB5B08DF-4A14-4273-9477-DF04FD94E411}" name="Table1" displayName="Table1" ref="A1:H4" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{AB5B08DF-4A14-4273-9477-DF04FD94E411}" name="Table1" displayName="Table1" ref="A1:H4" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="A1:H4" xr:uid="{AB5B08DF-4A14-4273-9477-DF04FD94E411}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -438,14 +475,14 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2C71C094-BA1E-42C2-BC6E-A0B697D5ABC9}" name="ลำดับที่" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{AEE929C0-CCBA-412E-863A-B93E45A6C76D}" name="รหัสนิสิต" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{D7AC4B30-710C-4DB3-A39A-82BE0E1CADB1}" name="ชื่อ-นามสกุล"/>
-    <tableColumn id="11" xr3:uid="{1A0F9857-0985-4CE6-A22D-59123392338B}" name="รหัสสาขา"/>
-    <tableColumn id="8" xr3:uid="{4D2CC8D0-C41F-424A-AFF5-4E7C19224356}" name="Email Google" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{E7F93D76-69FD-41A9-876B-E4FE9656B444}" name="คะแนนระหว่างเรียน"/>
-    <tableColumn id="5" xr3:uid="{EDFE6B02-7236-44AE-9510-F7331360E247}" name="คะแนนกลางภาค"/>
-    <tableColumn id="6" xr3:uid="{864306E6-76D3-4D83-ADF6-4D29F63A3522}" name="คะแนนปลายภาค"/>
+    <tableColumn id="1" xr3:uid="{2C71C094-BA1E-42C2-BC6E-A0B697D5ABC9}" name="ลำดับที่" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{AEE929C0-CCBA-412E-863A-B93E45A6C76D}" name="รหัสนิสิต" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{D7AC4B30-710C-4DB3-A39A-82BE0E1CADB1}" name="ชื่อ-นามสกุล" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{1A0F9857-0985-4CE6-A22D-59123392338B}" name="รหัสสาขา" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{4D2CC8D0-C41F-424A-AFF5-4E7C19224356}" name="Email Google" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{E7F93D76-69FD-41A9-876B-E4FE9656B444}" name="คะแนนระหว่างเรียน" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{EDFE6B02-7236-44AE-9510-F7331360E247}" name="คะแนนกลางภาค" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{864306E6-76D3-4D83-ADF6-4D29F63A3522}" name="คะแนนปลายภาค" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -771,13 +808,15 @@
   <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" customWidth="1"/>
-    <col min="3" max="3" width="30.5546875" customWidth="1"/>
-    <col min="5" max="5" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="30.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8.88671875" style="1"/>
+    <col min="5" max="5" width="18.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
@@ -807,82 +846,83 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="5">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="1">
         <v>20.5</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="1">
         <v>28.75</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-      <c r="M3" s="7"/>
-      <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
+      <c r="A4" s="6">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="1">
         <v>25.25</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="2">
     <mergeCell ref="J3:O3"/>
     <mergeCell ref="J2:O2"/>

</xml_diff>